<commit_message>
Reduce bolt geom inputs
</commit_message>
<xml_diff>
--- a/src/cassy/additional_data/templates/bolts/M12_bolt.xlsx
+++ b/src/cassy/additional_data/templates/bolts/M12_bolt.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DATA\laghida\Documents\GitLab\cassy\tests\runners\bolts\geometries\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\laghida\Documents\Github\cassy\src\cassy\additional_data\templates\bolts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67637075-426D-4282-83E6-CAEC54D40AC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E660137-AF57-4982-9B83-B27782065F96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2340" yWindow="2340" windowWidth="21600" windowHeight="11385" xr2:uid="{F09436F1-1F29-42A5-B1F9-53A78950820F}"/>
+    <workbookView xWindow="57480" yWindow="-240" windowWidth="29040" windowHeight="15720" xr2:uid="{F09436F1-1F29-42A5-B1F9-53A78950820F}"/>
   </bookViews>
   <sheets>
     <sheet name="Bolt Data" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="45">
   <si>
     <t>Dimensions of the bolts and assembled parts</t>
   </si>
@@ -63,9 +63,6 @@
   </si>
   <si>
     <t>d</t>
-  </si>
-  <si>
-    <t>maximum diameter (nominale)</t>
   </si>
   <si>
     <r>
@@ -254,6 +251,12 @@
   <si>
     <t>Inconel 718 (non leak tight) SDC-IC</t>
   </si>
+  <si>
+    <t>maximum diameter (nominal)</t>
+  </si>
+  <si>
+    <t>Only parameters in blue are mandatory. If the others are not provided (i.e., left empty) they will be computed according to ISO metric.</t>
+  </si>
 </sst>
 </file>
 
@@ -262,7 +265,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -316,6 +319,12 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -692,7 +701,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -810,6 +819,15 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="2" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="2" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -839,9 +857,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>169601</xdr:colOff>
-      <xdr:row>23</xdr:row>
-      <xdr:rowOff>20298</xdr:rowOff>
+      <xdr:colOff>172321</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>21425</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -883,9 +901,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>168954</xdr:colOff>
+      <xdr:colOff>171674</xdr:colOff>
       <xdr:row>26</xdr:row>
-      <xdr:rowOff>125625</xdr:rowOff>
+      <xdr:rowOff>121539</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -927,7 +945,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>24</xdr:col>
-      <xdr:colOff>207186</xdr:colOff>
+      <xdr:colOff>209908</xdr:colOff>
       <xdr:row>60</xdr:row>
       <xdr:rowOff>152400</xdr:rowOff>
     </xdr:to>
@@ -971,9 +989,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>515983</xdr:colOff>
+      <xdr:colOff>359361</xdr:colOff>
       <xdr:row>60</xdr:row>
-      <xdr:rowOff>164265</xdr:rowOff>
+      <xdr:rowOff>160179</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1307,16 +1325,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A35CF97-1329-4AF8-AE95-32CC01118615}">
   <dimension ref="A1:K25"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.84375" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="12.5703125" style="2" customWidth="1"/>
+    <col min="1" max="1" width="12.53515625" style="2" customWidth="1"/>
     <col min="2" max="2" width="44" style="2" customWidth="1"/>
-    <col min="3" max="3" width="26.7109375" style="2" customWidth="1"/>
-    <col min="4" max="11" width="11.140625" style="2" customWidth="1"/>
-    <col min="12" max="16384" width="8.85546875" style="2"/>
+    <col min="3" max="3" width="28.84375" style="2" customWidth="1"/>
+    <col min="4" max="11" width="11.15234375" style="2" customWidth="1"/>
+    <col min="12" max="16384" width="8.84375" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A1" s="37" t="s">
         <v>0</v>
       </c>
@@ -1331,7 +1349,7 @@
       <c r="J1" s="1"/>
       <c r="K1" s="1"/>
     </row>
-    <row r="2" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A2" s="10" t="s">
         <v>1</v>
       </c>
@@ -1352,7 +1370,7 @@
       <c r="J2" s="1"/>
       <c r="K2" s="1"/>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A3" s="14" t="s">
         <v>5</v>
       </c>
@@ -1373,12 +1391,12 @@
       <c r="J3" s="1"/>
       <c r="K3" s="1"/>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A4" s="3" t="s">
         <v>8</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>9</v>
+        <v>43</v>
       </c>
       <c r="C4" s="30">
         <v>12</v>
@@ -1394,15 +1412,15 @@
       <c r="J4" s="1"/>
       <c r="K4" s="1"/>
     </row>
-    <row r="5" spans="1:11" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" ht="16.75" x14ac:dyDescent="0.4">
       <c r="A5" s="3" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="C5" s="30">
-        <v>11.73</v>
+        <v>20</v>
+      </c>
+      <c r="C5" s="31">
+        <v>60</v>
       </c>
       <c r="D5" s="5" t="s">
         <v>7</v>
@@ -1415,18 +1433,17 @@
       <c r="J5" s="1"/>
       <c r="K5" s="1"/>
     </row>
-    <row r="6" spans="1:11" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="C6" s="30">
-        <f>C4</f>
-        <v>12</v>
-      </c>
-      <c r="D6" s="5" t="s">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A6" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="C6" s="31">
+        <v>0</v>
+      </c>
+      <c r="D6" s="9" t="s">
         <v>7</v>
       </c>
       <c r="E6" s="1"/>
@@ -1437,17 +1454,17 @@
       <c r="J6" s="1"/>
       <c r="K6" s="1"/>
     </row>
-    <row r="7" spans="1:11" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="C7" s="30">
-        <v>12</v>
-      </c>
-      <c r="D7" s="5" t="s">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A7" s="24" t="s">
+        <v>32</v>
+      </c>
+      <c r="B7" s="25" t="s">
+        <v>36</v>
+      </c>
+      <c r="C7" s="32">
+        <v>0</v>
+      </c>
+      <c r="D7" s="23" t="s">
         <v>7</v>
       </c>
       <c r="E7" s="1"/>
@@ -1458,17 +1475,17 @@
       <c r="J7" s="1"/>
       <c r="K7" s="1"/>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A8" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="C8" s="31">
-        <v>11.43</v>
-      </c>
-      <c r="D8" s="5" t="s">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A8" s="33" t="s">
+        <v>41</v>
+      </c>
+      <c r="B8" s="34" t="s">
+        <v>40</v>
+      </c>
+      <c r="C8" s="35">
+        <v>0</v>
+      </c>
+      <c r="D8" s="36" t="s">
         <v>7</v>
       </c>
       <c r="E8" s="1"/>
@@ -1479,17 +1496,14 @@
       <c r="J8" s="1"/>
       <c r="K8" s="1"/>
     </row>
-    <row r="9" spans="1:11" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" ht="16.75" x14ac:dyDescent="0.4">
       <c r="A9" s="3" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="C9" s="31">
-        <f>C4+1</f>
-        <v>13</v>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="C9" s="40"/>
       <c r="D9" s="5" t="s">
         <v>7</v>
       </c>
@@ -1501,16 +1515,14 @@
       <c r="J9" s="1"/>
       <c r="K9" s="1"/>
     </row>
-    <row r="10" spans="1:11" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" ht="16.75" x14ac:dyDescent="0.4">
       <c r="A10" s="3" t="s">
-        <v>36</v>
+        <v>11</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="C10" s="30">
-        <v>13.7</v>
-      </c>
+        <v>12</v>
+      </c>
+      <c r="C10" s="40"/>
       <c r="D10" s="5" t="s">
         <v>7</v>
       </c>
@@ -1522,16 +1534,14 @@
       <c r="J10" s="1"/>
       <c r="K10" s="1"/>
     </row>
-    <row r="11" spans="1:11" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" ht="16.75" x14ac:dyDescent="0.4">
       <c r="A11" s="3" t="s">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="C11" s="31">
-        <v>60</v>
-      </c>
+        <v>14</v>
+      </c>
+      <c r="C11" s="40"/>
       <c r="D11" s="5" t="s">
         <v>7</v>
       </c>
@@ -1543,16 +1553,14 @@
       <c r="J11" s="1"/>
       <c r="K11" s="1"/>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A12" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="B12" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="C12" s="31">
-        <v>6</v>
-      </c>
+        <v>15</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C12" s="41"/>
       <c r="D12" s="5" t="s">
         <v>7</v>
       </c>
@@ -1564,16 +1572,14 @@
       <c r="J12" s="1"/>
       <c r="K12" s="1"/>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" ht="16.75" x14ac:dyDescent="0.4">
       <c r="A13" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="B13" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="C13" s="31">
+        <v>17</v>
+      </c>
+      <c r="B13" s="4" t="s">
         <v>18</v>
       </c>
+      <c r="C13" s="41"/>
       <c r="D13" s="5" t="s">
         <v>7</v>
       </c>
@@ -1585,17 +1591,15 @@
       <c r="J13" s="1"/>
       <c r="K13" s="1"/>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A14" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="B14" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="C14" s="31">
-        <v>0</v>
-      </c>
-      <c r="D14" s="9" t="s">
+    <row r="14" spans="1:11" ht="16.75" x14ac:dyDescent="0.4">
+      <c r="A14" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="C14" s="40"/>
+      <c r="D14" s="5" t="s">
         <v>7</v>
       </c>
       <c r="E14" s="1"/>
@@ -1606,17 +1610,15 @@
       <c r="J14" s="1"/>
       <c r="K14" s="1"/>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A15" s="24" t="s">
-        <v>33</v>
-      </c>
-      <c r="B15" s="25" t="s">
-        <v>37</v>
-      </c>
-      <c r="C15" s="32">
-        <v>0</v>
-      </c>
-      <c r="D15" s="23" t="s">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A15" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="C15" s="41"/>
+      <c r="D15" s="5" t="s">
         <v>7</v>
       </c>
       <c r="E15" s="1"/>
@@ -1627,17 +1629,15 @@
       <c r="J15" s="1"/>
       <c r="K15" s="1"/>
     </row>
-    <row r="16" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="33" t="s">
-        <v>42</v>
-      </c>
-      <c r="B16" s="34" t="s">
-        <v>41</v>
-      </c>
-      <c r="C16" s="35">
-        <v>0</v>
-      </c>
-      <c r="D16" s="36" t="s">
+    <row r="16" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A16" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="C16" s="41"/>
+      <c r="D16" s="5" t="s">
         <v>7</v>
       </c>
       <c r="E16" s="1"/>
@@ -1648,18 +1648,18 @@
       <c r="J16" s="1"/>
       <c r="K16" s="1"/>
     </row>
-    <row r="17" spans="1:11" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" ht="16.75" x14ac:dyDescent="0.4">
       <c r="A17" s="26" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B17" s="27" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C17" s="16">
         <v>4</v>
       </c>
       <c r="D17" s="28" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E17" s="1"/>
       <c r="F17" s="1"/>
@@ -1669,18 +1669,18 @@
       <c r="J17" s="1"/>
       <c r="K17" s="1"/>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A18" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B18" s="6" t="s">
         <v>30</v>
-      </c>
-      <c r="B18" s="6" t="s">
-        <v>31</v>
       </c>
       <c r="C18" s="18">
         <v>0.15</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E18" s="1"/>
       <c r="F18" s="1"/>
@@ -1690,18 +1690,18 @@
       <c r="J18" s="1"/>
       <c r="K18" s="1"/>
     </row>
-    <row r="19" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A19" s="19" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B19" s="20" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C19" s="21">
         <v>0.15</v>
       </c>
       <c r="D19" s="22" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E19" s="1"/>
       <c r="F19" s="1"/>
@@ -1711,18 +1711,18 @@
       <c r="J19" s="1"/>
       <c r="K19" s="1"/>
     </row>
-    <row r="20" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A20" s="19" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B20" s="20" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C20" s="21" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D20" s="22" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E20" s="1"/>
       <c r="F20" s="1"/>
@@ -1732,7 +1732,7 @@
       <c r="J20" s="1"/>
       <c r="K20" s="1"/>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A21" s="1"/>
       <c r="B21" s="1"/>
       <c r="C21" s="1"/>
@@ -1745,11 +1745,13 @@
       <c r="J21" s="1"/>
       <c r="K21" s="1"/>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A22" s="1"/>
-      <c r="B22" s="1"/>
-      <c r="C22" s="1"/>
-      <c r="D22" s="1"/>
+    <row r="22" spans="1:11" ht="28.3" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A22" s="42" t="s">
+        <v>44</v>
+      </c>
+      <c r="B22" s="42"/>
+      <c r="C22" s="42"/>
+      <c r="D22" s="42"/>
       <c r="E22" s="1"/>
       <c r="F22" s="1"/>
       <c r="G22" s="1"/>
@@ -1758,7 +1760,7 @@
       <c r="J22" s="1"/>
       <c r="K22" s="1"/>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A23" s="1"/>
       <c r="B23" s="1"/>
       <c r="C23" s="1"/>
@@ -1771,7 +1773,7 @@
       <c r="J23" s="1"/>
       <c r="K23" s="1"/>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A24" s="1"/>
       <c r="B24" s="1"/>
       <c r="C24" s="1"/>
@@ -1784,7 +1786,7 @@
       <c r="J24" s="1"/>
       <c r="K24" s="1"/>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A25" s="1"/>
       <c r="B25" s="1"/>
       <c r="C25" s="1"/>
@@ -1798,8 +1800,9 @@
       <c r="K25" s="1"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
     <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A22:D22"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -1819,15 +1822,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100EFE0C39B20CFE747B2EDBEF1A424A9C1" ma:contentTypeVersion="14" ma:contentTypeDescription="Creare un nuovo documento." ma:contentTypeScope="" ma:versionID="fc5d43efe255f0326fdf88779d9e8cc0">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="71e126cb-1963-4e7b-b13a-15d2f64f78e9" xmlns:ns3="f41f4605-e15c-4135-bd96-d3970596b173" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="c67b044c92a952204dd5da40bf3ff3c1" ns2:_="" ns3:_="">
     <xsd:import namespace="71e126cb-1963-4e7b-b13a-15d2f64f78e9"/>
@@ -2056,6 +2050,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B53875E3-DFDB-4F02-8AAC-AEAA1E089733}">
   <ds:schemaRefs>
@@ -2070,14 +2073,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7F460EF5-1FE2-485A-B28D-6307C5242F38}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4AD0DBB6-51A1-41E4-B899-7133D1D7DFCB}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2094,4 +2089,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7F460EF5-1FE2-485A-B28D-6307C5242F38}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>